<commit_message>
docs: LOGIC_SPEC-v1.2 — office vendor accounting and linkage
</commit_message>
<xml_diff>
--- a/LOGIC_SPEC-v1.xlsx
+++ b/LOGIC_SPEC-v1.xlsx
@@ -814,6 +814,8 @@
                                 ▼
                          Design Expense (excluded from supervision base)
 Office Cash ──office_expense──► Operating Costs / Sectors
+Office Vendor ──project_expense──► Office Income
+Office Vendor ──procurement──► Office Income
 Employee ──custody──► Project / Office expense
 Employee ──payroll──► Salary expense</t>
         </is>
@@ -980,11 +982,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
@@ -1080,51 +1082,63 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>`(Owner Deposits + Supervision Income) − (Office Expenses + Withdrawals)`</t>
+          <t>`(Owner Deposits + Supervision Income + Office Vendor Income) − (Office Expenses + Withdrawals)`</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Net salary</t>
+          <t>Office vendor income</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>`Base Salary − Deductions + Bonuses − Penalties`</t>
+          <t>`Σ paid_amount of project_expense/vendor_settlement where vendor.is_office = true`</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Custody remaining</t>
+          <t>Net salary</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>`Given − Returned`</t>
+          <t>`Base Salary − Deductions + Bonuses − Penalties`</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>Custody remaining</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>`Given − Returned`</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
           <t>Unpaid balance (row)</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>`Amount − Paid Amount`</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>---</t>
         </is>
@@ -1132,7 +1146,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1203,7 +1217,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Version: 1.1</t>
+          <t>Version: 1.2</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -1870,29 +1884,77 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>3.4 Office Vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>The system seeds one special vendor marked `is_office = true` (e.g. "مكتب سارة أبو العلا"). This vendor represents the office itself and can be used for:</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Project expenses where the office is the service provider.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Procurements where the office is the supplier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Office expenses linked to a vendor for traceability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Transactions linked to the office vendor are not included in vendor balances or top-vendor dashboards; instead, their paid amounts are treated as office income and appear in the office cash-flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="21">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A11:H11"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A21:H21"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A11:H11"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A19:H19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: v294 retention/holdback tracking + supervision period-close audit rows
</commit_message>
<xml_diff>
--- a/LOGIC_SPEC-v1.xlsx
+++ b/LOGIC_SPEC-v1.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -867,7 +867,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>1. Supervision treatment</t>
+          <t>1. Supervision treatment *(resolved in v294)*</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>- It is still not stored as a separate receivable row. Decision: should it appear as an auto-generated `project_deposit` or `income` transaction?</t>
+          <t>- Period-close creates a system-locked `supervision` transaction row as an audit snapshot. Live balances continue to compute supervision from expenses.</t>
         </is>
       </c>
     </row>
@@ -958,40 +958,54 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>6. Retention / holdback (ضمان الأعمال)</t>
+          <t>6. Retention / holdback (ضمان الأعمال) *(resolved in v294)*</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>- Not implemented. Decide whether retention should be a separate transaction type, a project-level field, or an invoice line-item deduction.</t>
+          <t>- Implemented as a project-level `retention_percentage` plus companion `retention_withheld` / `retention_released` transaction rows.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>7. Password-reset email delivery verification</t>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>- `retention_withheld` is auto-generated on each `project_deposit` when `retention_percentage &gt; 0`.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>- `retention_released` is created manually by an admin at project close-out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>7. Password-reset email delivery verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>- The new `admin_reset_password_email` RPC (v289) enqueues the email via `pg_net`. The RPC returns success immediately; actual Resend delivery status must be checked in Resend logs or `net._http_response`.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="21">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A11:H11"/>
@@ -1002,12 +1016,14 @@
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A21:H21"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A17:H17"/>
     <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A19:H19"/>
@@ -1022,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1062,123 +1078,147 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>`Deposits − Expenses − Supervision`</t>
+          <t>`Deposits − Expenses − Supervision − Retention Withheld + Retention Released`</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Client balance (all views)</t>
+          <t>Net usable deposit</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>`Σ(Deposits − Expenses − Supervision)`</t>
+          <t>`Deposits − Retention Withheld + Retention Released`</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Client supervision</t>
+          <t>Client balance (all views)</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>`Σ Project Supervision across all client projects`</t>
+          <t>`Σ(Deposits − Expenses − Supervision − Retention Withheld + Retention Released)`</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Supervision fee</t>
+          <t>Client supervision</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>`(Expenses − Design Expenses) × Supervision% / 100`</t>
+          <t>`Σ Project Supervision across all client projects`</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Vendor balance</t>
+          <t>Supervision fee</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>`(Service Owed + Merchandise Owed) − (Direct Settlement Paid + Merchandise Paid)`</t>
+          <t>`(Expenses − Design Expenses) × Supervision% / 100`</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Office balance</t>
+          <t>Retained amount</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>`(Owner Deposits + Supervision Income + Office Vendor Income) − (Office Expenses + Withdrawals)`</t>
+          <t>`Deposit × Retention% / 100`</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Office vendor income</t>
+          <t>Vendor balance</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>`Σ vendor_settlement paid_amount + Σ procurement paid_amount where vendor.is_office = true`</t>
+          <t>`(Service Owed + Merchandise Owed) − (Direct Settlement Paid + Merchandise Paid)`</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Net salary</t>
+          <t>Office balance</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>`Base Salary − Deductions + Bonuses − Penalties`</t>
+          <t>`(Owner Deposits + Supervision Income + Office Vendor Income) − (Office Expenses + Withdrawals)`</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Custody remaining</t>
+          <t>Office vendor income</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>`Given − Returned`</t>
+          <t>`Σ vendor_settlement paid_amount + Σ procurement paid_amount where vendor.is_office = true`</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
+          <t>Net salary</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>`Base Salary − Deductions + Bonuses − Penalties`</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Custody remaining</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>`Given − Returned`</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
           <t>Unpaid balance (row)</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>`Amount − Paid Amount`</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>---</t>
         </is>
@@ -1186,7 +1226,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1632,7 +1672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -1669,137 +1709,155 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Project Deposits  = Σ Amount of all project_deposit transactions
-Project Expenses  = Σ Amount of all project_expense transactions
-Design Expenses   = Σ Amount of project_expense where category = design
-Construction Exp. = Project Expenses − Design Expenses</t>
+          <t>Project Deposits      = Σ Amount of all project_deposit transactions
+Project Expenses      = Σ Amount of all project_expense transactions
+Design Expenses       = Σ Amount of project_expense where category = design
+Construction Exp.     = Project Expenses − Design Expenses
+Retention Withheld    = Σ Amount of retention_withheld transactions
+Retention Released    = Σ Amount of retention_released transactions</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>`Retention %` is stored on the project master record. When a `project_deposit` is saved and `Retention % &gt; 0`, a companion `retention_withheld` row is auto-generated for `Deposit × Retention %`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>2.2 Supervision Fee</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Supervision is a fee the office earns as a percentage of construction-related expenses only. Design costs are excluded from the base.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Supervision Fee = Construction Expenses × (Supervision % / 100)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Where `Supervision %` is set on the project master record.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Important: Supervision is computed on demand and is not stored as a separate transaction row. It affects project net balance and office income, but it does not appear directly in the transaction list unless a manual supervision transaction is created.</t>
-        </is>
-      </c>
-    </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Live supervision is computed on demand and affects project net balance and office income. When an admin closes a project period, a `system_generated = true` `supervision` transaction row is created as an immutable audit snapshot for that period. This stored row is excluded from live supervision totals to avoid double counting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>2.3 Project Net Balance</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Project Net Balance = Project Deposits − Project Expenses − Supervision Fee</t>
-        </is>
-      </c>
-    </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Project Net Balance = Project Deposits − Project Expenses − Supervision Fee − Retention Withheld + Retention Released</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>`Net Usable Deposit = Project Deposits − Retention Withheld + Retention Released`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Interpretation:</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Positive → client still owes money (deposits exceed costs + fee).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Zero → account is square.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Negative → project is over-budget or over-paid by the client.</t>
+          <t>Positive → client still owes money (deposits exceed costs + fee).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>Zero → account is square.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Negative → project is over-budget or over-paid by the client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>Project expenses are treated as fully paid. The `paid_amount` field is not collected on the project expense form; `paid_amount` is set equal to `amount` and `payment_term` is set to `immediate`. Any subsequent payment to the vendor is recorded separately as a project-agnostic `vendor_settlement` from the vendors screen.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>2.4 Client Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>A client may have many projects. The client balance is the sum of the net balances of all client projects, with supervision applied consistently everywhere:</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Client Deposits    = Σ Project Deposits     (for all client projects)
-Client Expenses    = Σ Project Expenses     (for all client projects)
-Client Supervision = Σ Supervision Fee      (for all client projects)
-Client Balance     = Client Deposits − Client Expenses − Client Supervision</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>A client may have many projects. The client balance is the sum of the net balances of all client projects, with supervision and retention applied consistently everywhere:</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Client Deposits         = Σ Project Deposits       (for all client projects)
+Client Expenses         = Σ Project Expenses       (for all client projects)
+Client Supervision      = Σ Supervision Fee        (for all client projects)
+Client Retention Held   = Σ Retention Withheld     (for all client projects)
+Client Retention Released = Σ Retention Released   (for all client projects)
+Client Balance          = Client Deposits − Client Expenses − Client Supervision − Client Retention Held + Client Retention Released</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>The same supervision formula is applied consistently in project detail, client detail, client list, and dashboard active-client balances. The canonical view `client_balances` enforces this formula.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="23">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A11:H11"/>
@@ -1814,7 +1872,9 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A23:H23"/>
     <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A22:H22"/>
     <mergeCell ref="A17:H17"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A20:H20"/>

</xml_diff>